<commit_message>
Add validation models ml
</commit_message>
<xml_diff>
--- a/data/out/best_models_lstm/best_lstm_metrics.xlsx
+++ b/data/out/best_models_lstm/best_lstm_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,7 +541,938 @@
         <v>9634</v>
       </c>
       <c r="M2" t="n">
-        <v>140.0892918109894</v>
+        <v>156.7648313045502</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>v1_original_lags</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.8840208649635315</v>
+      </c>
+      <c r="E3" t="n">
+        <v>82.96078491210938</v>
+      </c>
+      <c r="F3" t="n">
+        <v>29174.2421875</v>
+      </c>
+      <c r="G3" t="n">
+        <v>170.8046875</v>
+      </c>
+      <c r="H3" t="n">
+        <v>21.72550857067108</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>48144</v>
+      </c>
+      <c r="K3" t="n">
+        <v>38515</v>
+      </c>
+      <c r="L3" t="n">
+        <v>9629</v>
+      </c>
+      <c r="M3" t="n">
+        <v>154.1242589950562</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>v2_with_calendar</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.4815700054168701</v>
+      </c>
+      <c r="E4" t="n">
+        <v>211.3009490966797</v>
+      </c>
+      <c r="F4" t="n">
+        <v>130342.3203125</v>
+      </c>
+      <c r="G4" t="n">
+        <v>361.029541015625</v>
+      </c>
+      <c r="H4" t="n">
+        <v>38.82325887680054</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K4" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L4" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M4" t="n">
+        <v>140.4664907455444</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>v2_with_calendar_lags</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.8731307983398438</v>
+      </c>
+      <c r="E5" t="n">
+        <v>84.36554718017578</v>
+      </c>
+      <c r="F5" t="n">
+        <v>31913.607421875</v>
+      </c>
+      <c r="G5" t="n">
+        <v>178.643798828125</v>
+      </c>
+      <c r="H5" t="n">
+        <v>20.5694779753685</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>48144</v>
+      </c>
+      <c r="K5" t="n">
+        <v>38515</v>
+      </c>
+      <c r="L5" t="n">
+        <v>9629</v>
+      </c>
+      <c r="M5" t="n">
+        <v>153.152601480484</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>v3_no_solar</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.4528739452362061</v>
+      </c>
+      <c r="E6" t="n">
+        <v>221.0094146728516</v>
+      </c>
+      <c r="F6" t="n">
+        <v>137557</v>
+      </c>
+      <c r="G6" t="n">
+        <v>370.8867797851562</v>
+      </c>
+      <c r="H6" t="n">
+        <v>38.89133334159851</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K6" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L6" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M6" t="n">
+        <v>145.9975438117981</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>v3_no_solar_lags</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.8539999723434448</v>
+      </c>
+      <c r="E7" t="n">
+        <v>93.26525115966797</v>
+      </c>
+      <c r="F7" t="n">
+        <v>36725.91796875</v>
+      </c>
+      <c r="G7" t="n">
+        <v>191.6400756835938</v>
+      </c>
+      <c r="H7" t="n">
+        <v>20.06335556507111</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>48144</v>
+      </c>
+      <c r="K7" t="n">
+        <v>38515</v>
+      </c>
+      <c r="L7" t="n">
+        <v>9629</v>
+      </c>
+      <c r="M7" t="n">
+        <v>150.2669422626495</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>v4_no_fuel_consumption</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.347089409828186</v>
+      </c>
+      <c r="E8" t="n">
+        <v>233.6261901855469</v>
+      </c>
+      <c r="F8" t="n">
+        <v>164153.078125</v>
+      </c>
+      <c r="G8" t="n">
+        <v>405.1580810546875</v>
+      </c>
+      <c r="H8" t="n">
+        <v>39.42742943763733</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K8" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L8" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M8" t="n">
+        <v>138.7522842884064</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>v4_no_fuel_consumption_lags</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.8692944049835205</v>
+      </c>
+      <c r="E9" t="n">
+        <v>86.45876312255859</v>
+      </c>
+      <c r="F9" t="n">
+        <v>32878.63671875</v>
+      </c>
+      <c r="G9" t="n">
+        <v>181.3246765136719</v>
+      </c>
+      <c r="H9" t="n">
+        <v>19.96601521968842</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>48144</v>
+      </c>
+      <c r="K9" t="n">
+        <v>38515</v>
+      </c>
+      <c r="L9" t="n">
+        <v>9629</v>
+      </c>
+      <c r="M9" t="n">
+        <v>139.9519515037537</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>v5_no_fuel_and_cost</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.3703179955482483</v>
+      </c>
+      <c r="E10" t="n">
+        <v>227.6237335205078</v>
+      </c>
+      <c r="F10" t="n">
+        <v>158313.015625</v>
+      </c>
+      <c r="G10" t="n">
+        <v>397.8856811523438</v>
+      </c>
+      <c r="H10" t="n">
+        <v>46.5480238199234</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K10" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L10" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M10" t="n">
+        <v>82.00382661819458</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>v5_no_fuel_and_cost_lags</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.8767141699790955</v>
+      </c>
+      <c r="E11" t="n">
+        <v>84.22475433349609</v>
+      </c>
+      <c r="F11" t="n">
+        <v>31012.21484375</v>
+      </c>
+      <c r="G11" t="n">
+        <v>176.1028594970703</v>
+      </c>
+      <c r="H11" t="n">
+        <v>19.53263580799103</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>48144</v>
+      </c>
+      <c r="K11" t="n">
+        <v>38515</v>
+      </c>
+      <c r="L11" t="n">
+        <v>9629</v>
+      </c>
+      <c r="M11" t="n">
+        <v>71.68802714347839</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>v6_no_econ_fuel_cost</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.08480823040008545</v>
+      </c>
+      <c r="E12" t="n">
+        <v>285.0439453125</v>
+      </c>
+      <c r="F12" t="n">
+        <v>230095.140625</v>
+      </c>
+      <c r="G12" t="n">
+        <v>479.6823425292969</v>
+      </c>
+      <c r="H12" t="n">
+        <v>48.03547561168671</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K12" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L12" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M12" t="n">
+        <v>70.71074938774109</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>v6_no_econ_fuel_cost_lags</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.8569105863571167</v>
+      </c>
+      <c r="E13" t="n">
+        <v>94.25941467285156</v>
+      </c>
+      <c r="F13" t="n">
+        <v>35993.76171875</v>
+      </c>
+      <c r="G13" t="n">
+        <v>189.72021484375</v>
+      </c>
+      <c r="H13" t="n">
+        <v>21.67570888996124</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>48144</v>
+      </c>
+      <c r="K13" t="n">
+        <v>38515</v>
+      </c>
+      <c r="L13" t="n">
+        <v>9629</v>
+      </c>
+      <c r="M13" t="n">
+        <v>73.32901000976562</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>lstm_bidirectional</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>v7_only_gen_enso</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.3108968734741211</v>
+      </c>
+      <c r="E14" t="n">
+        <v>225.3665466308594</v>
+      </c>
+      <c r="F14" t="n">
+        <v>173252.515625</v>
+      </c>
+      <c r="G14" t="n">
+        <v>416.2361145019531</v>
+      </c>
+      <c r="H14" t="n">
+        <v>53.87526154518127</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K14" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L14" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M14" t="n">
+        <v>406.1756017208099</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>bilstm_stacked</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>v7_only_gen_enso_lags</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.2985653281211853</v>
+      </c>
+      <c r="E15" t="n">
+        <v>252.1846313476562</v>
+      </c>
+      <c r="F15" t="n">
+        <v>176352.890625</v>
+      </c>
+      <c r="G15" t="n">
+        <v>419.9439086914062</v>
+      </c>
+      <c r="H15" t="n">
+        <v>56.74571394920349</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K15" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L15" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1325.787066936493</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>bilstm_stacked</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>v8_only_gen_no_solar_enso</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.5544328689575195</v>
+      </c>
+      <c r="E16" t="n">
+        <v>176.4687957763672</v>
+      </c>
+      <c r="F16" t="n">
+        <v>112023.328125</v>
+      </c>
+      <c r="G16" t="n">
+        <v>334.6988525390625</v>
+      </c>
+      <c r="H16" t="n">
+        <v>47.4595695734024</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K16" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L16" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1376.884832382202</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>lstm_deep</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>v8_only_gen_no_solar_enso_lags</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.3108347058296204</v>
+      </c>
+      <c r="E17" t="n">
+        <v>228.9801940917969</v>
+      </c>
+      <c r="F17" t="n">
+        <v>173268.15625</v>
+      </c>
+      <c r="G17" t="n">
+        <v>416.2549133300781</v>
+      </c>
+      <c r="H17" t="n">
+        <v>46.74026370048523</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>48168</v>
+      </c>
+      <c r="K17" t="n">
+        <v>38534</v>
+      </c>
+      <c r="L17" t="n">
+        <v>9634</v>
+      </c>
+      <c r="M17" t="n">
+        <v>3955.097734689713</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>v9_date_range_all</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>-1.600795269012451</v>
+      </c>
+      <c r="E18" t="n">
+        <v>138.1423645019531</v>
+      </c>
+      <c r="F18" t="n">
+        <v>25089.265625</v>
+      </c>
+      <c r="G18" t="n">
+        <v>158.3959197998047</v>
+      </c>
+      <c r="H18" t="n">
+        <v>111.3688349723816</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>13081</v>
+      </c>
+      <c r="K18" t="n">
+        <v>10464</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2617</v>
+      </c>
+      <c r="M18" t="n">
+        <v>46.4168598651886</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>v9_date_range_all_lags</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.2878156304359436</v>
+      </c>
+      <c r="E19" t="n">
+        <v>49.89236831665039</v>
+      </c>
+      <c r="F19" t="n">
+        <v>6881.70849609375</v>
+      </c>
+      <c r="G19" t="n">
+        <v>82.95606231689453</v>
+      </c>
+      <c r="H19" t="n">
+        <v>34.83904898166656</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>13057</v>
+      </c>
+      <c r="K19" t="n">
+        <v>10445</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2612</v>
+      </c>
+      <c r="M19" t="n">
+        <v>38.82591557502747</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>lstm_simple</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>v10_date_range_no_solar</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.7960166931152344</v>
+      </c>
+      <c r="E20" t="n">
+        <v>117.7841033935547</v>
+      </c>
+      <c r="F20" t="n">
+        <v>17325.75390625</v>
+      </c>
+      <c r="G20" t="n">
+        <v>131.6273345947266</v>
+      </c>
+      <c r="H20" t="n">
+        <v>93.74042749404907</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>13081</v>
+      </c>
+      <c r="K20" t="n">
+        <v>10464</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2617</v>
+      </c>
+      <c r="M20" t="n">
+        <v>110.4701633453369</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LSTM</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>cnn_lstm</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>v10_date_range_no_solar_lags</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.2673751711845398</v>
+      </c>
+      <c r="E21" t="n">
+        <v>53.41995620727539</v>
+      </c>
+      <c r="F21" t="n">
+        <v>7079.220703125</v>
+      </c>
+      <c r="G21" t="n">
+        <v>84.13810729980469</v>
+      </c>
+      <c r="H21" t="n">
+        <v>38.23941051959991</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>trained</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>13057</v>
+      </c>
+      <c r="K21" t="n">
+        <v>10445</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2612</v>
+      </c>
+      <c r="M21" t="n">
+        <v>41.35307002067566</v>
       </c>
     </row>
   </sheetData>

</xml_diff>